<commit_message>
Implementasikan pengingat jurnal dengan mengirim pesan WhatsApp kepada dosen
</commit_message>
<xml_diff>
--- a/public/templates/bahan_import_template.xlsx
+++ b/public/templates/bahan_import_template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="21">
   <si>
     <t>kode</t>
   </si>
@@ -46,6 +46,9 @@
   </si>
   <si>
     <t>Laboratorium Komputer ICT Lantai 1</t>
+  </si>
+  <si>
+    <t>tanggal_kedaluwarsa</t>
   </si>
   <si>
     <t>Laboratorium Analisis Zat Gizi</t>
@@ -431,17 +434,17 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="9.283" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="8.141" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="8.141" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="41.133" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="9.283" customWidth="true" style="0"/>
+    <col min="2" max="2" width="12.854" customWidth="true" style="0"/>
+    <col min="3" max="3" width="8.141" customWidth="true" style="0"/>
+    <col min="4" max="4" width="8.141" customWidth="true" style="0"/>
+    <col min="5" max="5" width="41.133" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -457,8 +460,11 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -499,7 +505,7 @@
   <dimension ref="A1:A12"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="41.133" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="41.133" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
@@ -509,17 +515,17 @@
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:1">
@@ -529,37 +535,37 @@
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>